<commit_message>
Barefoot draft: updated PDF (value-first, payment terms) and cover note
Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01F75G8iv8ooxhkGc1PV5mNB
</commit_message>
<xml_diff>
--- a/sales-engine/customers/elephant-barefoot-lodge/Barefoot_5Year_Business_Case.xlsx
+++ b/sales-engine/customers/elephant-barefoot-lodge/Barefoot_5Year_Business_Case.xlsx
@@ -2563,7 +2563,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:C29"/>
+  <dimension ref="A1:C32"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15" outlineLevelCol="0"/>
   <cols>
     <col width="3" customWidth="1" min="1" max="1"/>
@@ -2639,178 +2639,229 @@
     <row r="7" ht="30" customHeight="1">
       <c r="A7" s="5" t="inlineStr">
         <is>
-          <t>Timing of the comparison</t>
+          <t>Payment terms - build</t>
         </is>
       </c>
       <c r="B7" s="17" t="inlineStr">
         <is>
-          <t>Both paths start at month 1</t>
+          <t>50% deposit on order, 50% on commissioning</t>
         </is>
       </c>
       <c r="C7" s="32" t="inlineStr">
         <is>
-          <t>Year 0 is the build payment only. Neither path is charged any monthly bill in year 0 - an earlier version of this model charged Herotel a full year before the build and gave the CTTX path none, which overstated the case. Corrected 28 Sept 2026.</t>
+          <t>The deposit places the equipment order and secures the allocation. Both halves fall in year 0 of the cash flow, so the model is unchanged by the split.</t>
         </is>
       </c>
     </row>
     <row r="8" ht="30" customHeight="1">
       <c r="A8" s="5" t="inlineStr">
         <is>
-          <t>VAT rate</t>
+          <t>Accounting treatment - build</t>
         </is>
       </c>
       <c r="B8" s="17" t="inlineStr">
         <is>
-          <t>15%</t>
+          <t>Capital expenditure (fixed asset)</t>
         </is>
       </c>
       <c r="C8" s="32" t="inlineStr">
         <is>
-          <t>Current South African VAT rate.</t>
+          <t>R308,696 ex VAT is capitalised as owned infrastructure on the lodge's balance sheet; the R46,304 input VAT is recoverable for a VAT-registered entity; the asset is depreciable over its working life and transfers with the property. The lodge's accountant confirms the exact treatment - this workbook does not model the tax effect (which would only improve the case).</t>
         </is>
       </c>
     </row>
     <row r="9" ht="30" customHeight="1">
       <c r="A9" s="5" t="inlineStr">
         <is>
-          <t>Managed Service Retainer</t>
+          <t>Spa and future endpoints</t>
         </is>
       </c>
       <c r="B9" s="17" t="inlineStr">
         <is>
-          <t>R1,500/month excl. VAT</t>
+          <t>Not in the current-provider line</t>
         </is>
       </c>
       <c r="C9" s="32" t="inlineStr">
         <is>
-          <t>Set by Gerhard (26 Sept 2026) - a lighter monthly retainer to keep the recurring bill low relative to Herotel and support the case for the build investment.</t>
+          <t>The current bill excludes the spa (not connected today). On the rental model each additional AP is ~R263/month incl. VAT (per the current invoice) plus a link to reach the spa; on the owned network it is a once-off hardware cost. Left out of the comparison deliberately - the current-provider line is therefore understated, not overstated.</t>
         </is>
       </c>
     </row>
     <row r="10" ht="30" customHeight="1">
       <c r="A10" s="5" t="inlineStr">
         <is>
+          <t>Timing of the comparison</t>
+        </is>
+      </c>
+      <c r="B10" s="17" t="inlineStr">
+        <is>
+          <t>Both paths start at month 1</t>
+        </is>
+      </c>
+      <c r="C10" s="32" t="inlineStr">
+        <is>
+          <t>Year 0 is the build payment only. Neither path is charged any monthly bill in year 0 - an earlier version of this model charged Herotel a full year before the build and gave the CTTX path none, which overstated the case. Corrected 28 Sept 2026.</t>
+        </is>
+      </c>
+    </row>
+    <row r="11" ht="30" customHeight="1">
+      <c r="A11" s="5" t="inlineStr">
+        <is>
+          <t>VAT rate</t>
+        </is>
+      </c>
+      <c r="B11" s="17" t="inlineStr">
+        <is>
+          <t>15%</t>
+        </is>
+      </c>
+      <c r="C11" s="32" t="inlineStr">
+        <is>
+          <t>Current South African VAT rate.</t>
+        </is>
+      </c>
+    </row>
+    <row r="12" ht="30" customHeight="1">
+      <c r="A12" s="5" t="inlineStr">
+        <is>
+          <t>Managed Service Retainer</t>
+        </is>
+      </c>
+      <c r="B12" s="17" t="inlineStr">
+        <is>
+          <t>R1,500/month excl. VAT</t>
+        </is>
+      </c>
+      <c r="C12" s="32" t="inlineStr">
+        <is>
+          <t>Set by Gerhard (26 Sept 2026) - a lighter monthly retainer to keep the recurring bill low relative to Herotel and support the case for the build investment.</t>
+        </is>
+      </c>
+    </row>
+    <row r="13" ht="30" customHeight="1">
+      <c r="A13" s="5" t="inlineStr">
+        <is>
           <t>Contract term - Vodacom Business Connect</t>
         </is>
       </c>
-      <c r="B10" s="17" t="inlineStr">
+      <c r="B13" s="17" t="inlineStr">
         <is>
           <t>36 months</t>
         </is>
       </c>
-      <c r="C10" s="32" t="inlineStr">
+      <c r="C13" s="32" t="inlineStr">
         <is>
           <t>Confirmed 28 Sept 2026 against the CTTX Vodacom Reseller price book (Duane Forlee, Vodacom, 29 May 2026): the 36-month rate is slightly lower than 24-month. Monthly figure in this model is the confirmed 36-month client price at CTTX's standard 20% markup.</t>
         </is>
       </c>
     </row>
-    <row r="12">
-      <c r="A12" s="9" t="inlineStr">
+    <row r="15">
+      <c r="A15" s="9" t="inlineStr">
         <is>
           <t>Design Assumptions</t>
-        </is>
-      </c>
-    </row>
-    <row r="13" ht="32" customHeight="1">
-      <c r="A13" s="32" t="inlineStr">
-        <is>
-          <t>Single 9m mast carrying two 90-degree sector antennas (confirmed by Gerhard, 26 Sept 2026) - replaces the lodge's existing leaning gum-pole mount. This is NOT a two-site build; earlier drafts of this costing incorrectly read the field survey's two radio labels as two separate physical locations before this was corrected.</t>
-        </is>
-      </c>
-    </row>
-    <row r="14" ht="32" customHeight="1">
-      <c r="A14" s="32" t="inlineStr">
-        <is>
-          <t>Line-of-sight confirmed for all 28 subscriber links by Abel Ringisai's field RF survey (KML export, 22 Sept 2026).</t>
-        </is>
-      </c>
-    </row>
-    <row r="15" ht="32" customHeight="1">
-      <c r="A15" s="32" t="inlineStr">
-        <is>
-          <t>The longest links (1.7km-3.0km, to the staff village and Director's House) sit at the edge of the serving sector's range and still need a link-budget check to confirm they sustain full 100 Mbps symmetrical - flagged, not yet resolved.</t>
         </is>
       </c>
     </row>
     <row r="16" ht="32" customHeight="1">
       <c r="A16" s="32" t="inlineStr">
         <is>
-          <t>Cable run priced at an average 40m per run - to be confirmed once exact distances are measured on site.</t>
+          <t>Single 9m mast carrying two 90-degree sector antennas (confirmed by Gerhard, 26 Sept 2026) - replaces the lodge's existing leaning gum-pole mount. This is NOT a two-site build; earlier drafts of this costing incorrectly read the field survey's two radio labels as two separate physical locations before this was corrected.</t>
         </is>
       </c>
     </row>
     <row r="17" ht="32" customHeight="1">
       <c r="A17" s="32" t="inlineStr">
         <is>
-          <t>Vodacom Business Connect feasibility for this specific site has not yet been formally submitted/approved.</t>
-        </is>
-      </c>
-    </row>
-    <row r="19">
-      <c r="A19" s="9" t="inlineStr">
-        <is>
-          <t>What's Included in the 10-Year Support</t>
+          <t>Line-of-sight confirmed for all 28 subscriber links by Abel Ringisai's field RF survey (KML export, 22 Sept 2026).</t>
+        </is>
+      </c>
+    </row>
+    <row r="18" ht="32" customHeight="1">
+      <c r="A18" s="32" t="inlineStr">
+        <is>
+          <t>The longest links (1.7km-3.0km, to the staff village and Director's House) sit at the edge of the serving sector's range and still need a link-budget check to confirm they sustain full 100 Mbps symmetrical - flagged, not yet resolved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="19" ht="32" customHeight="1">
+      <c r="A19" s="32" t="inlineStr">
+        <is>
+          <t>Cable run priced at an average 40m per run - to be confirmed once exact distances are measured on site.</t>
         </is>
       </c>
     </row>
     <row r="20" ht="32" customHeight="1">
       <c r="A20" s="32" t="inlineStr">
         <is>
+          <t>Vodacom Business Connect feasibility for this specific site has not yet been formally submitted/approved.</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="9" t="inlineStr">
+        <is>
+          <t>What's Included in the 10-Year Support</t>
+        </is>
+      </c>
+    </row>
+    <row r="23" ht="32" customHeight="1">
+      <c r="A23" s="32" t="inlineStr">
+        <is>
           <t>Years 1-3: monthly remote monitoring, quarterly on-site maintenance, 24/7 emergency support, proactive performance reporting, warranty-covered equipment troubleshooting/replacement.</t>
         </is>
       </c>
     </row>
-    <row r="21" ht="32" customHeight="1">
-      <c r="A21" s="32" t="inlineStr">
+    <row r="24" ht="32" customHeight="1">
+      <c r="A24" s="32" t="inlineStr">
         <is>
           <t>Years 4-10: ongoing remote monitoring, annual on-site maintenance/assessment, 24/7 support continuation, planned technology refresh, performance reporting.</t>
-        </is>
-      </c>
-    </row>
-    <row r="22" ht="32" customHeight="1">
-      <c r="A22" s="32" t="inlineStr">
-        <is>
-          <t>Throughout: no vendor lock-in on the owned hardware, scalability support, staff training and documentation.</t>
-        </is>
-      </c>
-    </row>
-    <row r="24">
-      <c r="A24" s="9" t="inlineStr">
-        <is>
-          <t>What's Excluded / Not Yet Priced</t>
         </is>
       </c>
     </row>
     <row r="25" ht="32" customHeight="1">
       <c r="A25" s="32" t="inlineStr">
         <is>
-          <t>Major component replacement (Lithium battery bank, inverter) near the end of the 10-year term - typical service life for this equipment is 8-10 years, so a replacement reserve may be needed in years 8-10 and is not included in the build cost above.</t>
-        </is>
-      </c>
-    </row>
-    <row r="26" ht="32" customHeight="1">
-      <c r="A26" s="32" t="inlineStr">
-        <is>
-          <t>Trenching or underground civil works (none required - this is a wireless solution).</t>
-        </is>
-      </c>
-    </row>
-    <row r="27" ht="32" customHeight="1">
-      <c r="A27" s="32" t="inlineStr">
-        <is>
-          <t>CCTV cameras, POS hardware, or other endpoint devices not listed in the hardware BOM.</t>
+          <t>Throughout: no vendor lock-in on the owned hardware, scalability support, staff training and documentation.</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="9" t="inlineStr">
+        <is>
+          <t>What's Excluded / Not Yet Priced</t>
         </is>
       </c>
     </row>
     <row r="28" ht="32" customHeight="1">
       <c r="A28" s="32" t="inlineStr">
         <is>
-          <t>Travel/accommodation beyond a day-trip assumption from Port Elizabeth (~1h45 drive) - to be confirmed if overnight stays are required during the 3-day install.</t>
+          <t>Major component replacement (Lithium battery bank, inverter) near the end of the 10-year term - typical service life for this equipment is 8-10 years, so a replacement reserve may be needed in years 8-10 and is not included in the build cost above.</t>
         </is>
       </c>
     </row>
     <row r="29" ht="32" customHeight="1">
       <c r="A29" s="32" t="inlineStr">
+        <is>
+          <t>Trenching or underground civil works (none required - this is a wireless solution).</t>
+        </is>
+      </c>
+    </row>
+    <row r="30" ht="32" customHeight="1">
+      <c r="A30" s="32" t="inlineStr">
+        <is>
+          <t>CCTV cameras, POS hardware, or other endpoint devices not listed in the hardware BOM.</t>
+        </is>
+      </c>
+    </row>
+    <row r="31" ht="32" customHeight="1">
+      <c r="A31" s="32" t="inlineStr">
+        <is>
+          <t>Travel/accommodation beyond a day-trip assumption from Port Elizabeth (~1h45 drive) - to be confirmed if overnight stays are required during the 3-day install.</t>
+        </is>
+      </c>
+    </row>
+    <row r="32" ht="32" customHeight="1">
+      <c r="A32" s="32" t="inlineStr">
         <is>
           <t>Any scope beyond the confirmed coverage zones (28 subscriber sites) without a signed change order.</t>
         </is>
@@ -2820,22 +2871,22 @@
   <mergeCells count="18">
     <mergeCell ref="A25:C25"/>
     <mergeCell ref="A28:C28"/>
-    <mergeCell ref="A13:C13"/>
     <mergeCell ref="A19:C19"/>
-    <mergeCell ref="A26:C26"/>
     <mergeCell ref="A1:C1"/>
-    <mergeCell ref="A14:C14"/>
+    <mergeCell ref="A23:C23"/>
+    <mergeCell ref="A32:C32"/>
+    <mergeCell ref="A31:C31"/>
     <mergeCell ref="A22:C22"/>
     <mergeCell ref="A17:C17"/>
+    <mergeCell ref="A18:C18"/>
     <mergeCell ref="A27:C27"/>
     <mergeCell ref="A3:C3"/>
-    <mergeCell ref="A21:C21"/>
-    <mergeCell ref="A12:C12"/>
+    <mergeCell ref="A30:C30"/>
+    <mergeCell ref="A15:C15"/>
     <mergeCell ref="A20:C20"/>
     <mergeCell ref="A24:C24"/>
     <mergeCell ref="A16:C16"/>
     <mergeCell ref="A29:C29"/>
-    <mergeCell ref="A15:C15"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>